<commit_message>
feat: do more analysis about the rosemary datasets in endosome
</commit_message>
<xml_diff>
--- a/data/proteomics/membrane_size_across_compartment_tao2.xlsx
+++ b/data/proteomics/membrane_size_across_compartment_tao2.xlsx
@@ -485,28 +485,28 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>236.8128453591501</v>
+        <v>236.8128453591497</v>
       </c>
       <c r="D2" t="n">
-        <v>245.3879189787729</v>
+        <v>245.3879189787723</v>
       </c>
       <c r="E2" t="n">
-        <v>112.5722153668912</v>
+        <v>112.5722153668911</v>
       </c>
       <c r="F2" t="n">
         <v>132.4842566734899</v>
       </c>
       <c r="G2" t="n">
-        <v>176.0780151840229</v>
+        <v>176.0780151840232</v>
       </c>
       <c r="H2" t="n">
-        <v>182.5266953598283</v>
+        <v>182.5266953598284</v>
       </c>
       <c r="I2" t="n">
-        <v>106.4375502663249</v>
+        <v>106.437550266325</v>
       </c>
       <c r="J2" t="n">
-        <v>114.5350118663038</v>
+        <v>114.5350118663039</v>
       </c>
     </row>
     <row r="3">
@@ -522,7 +522,7 @@
         <v>0.6100240646422364</v>
       </c>
       <c r="D3" t="n">
-        <v>0.730011269698384</v>
+        <v>0.7300112696983838</v>
       </c>
       <c r="E3" t="n">
         <v>0.2602091706226773</v>
@@ -534,13 +534,13 @@
         <v>0.58627600929545</v>
       </c>
       <c r="H3" t="n">
-        <v>0.5958036382317059</v>
+        <v>0.595803638231706</v>
       </c>
       <c r="I3" t="n">
-        <v>0.3550735645846797</v>
+        <v>0.3550735645846796</v>
       </c>
       <c r="J3" t="n">
-        <v>0.3950978682794314</v>
+        <v>0.3950978682794315</v>
       </c>
     </row>
     <row r="4">
@@ -553,25 +553,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.9399759257931882</v>
+        <v>0.939975925793188</v>
       </c>
       <c r="D4" t="n">
         <v>1.033371901011972</v>
       </c>
       <c r="E4" t="n">
-        <v>0.4708206233552723</v>
+        <v>0.4708206233552722</v>
       </c>
       <c r="F4" t="n">
-        <v>0.716776490061686</v>
+        <v>0.7167764900616861</v>
       </c>
       <c r="G4" t="n">
         <v>0.9261789993993077</v>
       </c>
       <c r="H4" t="n">
-        <v>0.940250115699143</v>
+        <v>0.9402501156991431</v>
       </c>
       <c r="I4" t="n">
-        <v>0.549744225627545</v>
+        <v>0.5497442256275451</v>
       </c>
       <c r="J4" t="n">
         <v>0.5708457638205316</v>
@@ -621,28 +621,28 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>94.08831465042724</v>
+        <v>94.08831465042711</v>
       </c>
       <c r="D6" t="n">
         <v>100.3359130541194</v>
       </c>
       <c r="E6" t="n">
-        <v>59.17422201776203</v>
+        <v>59.17422201776201</v>
       </c>
       <c r="F6" t="n">
-        <v>71.13413790398974</v>
+        <v>71.13413790398985</v>
       </c>
       <c r="G6" t="n">
-        <v>88.40347857667676</v>
+        <v>88.40347857667683</v>
       </c>
       <c r="H6" t="n">
-        <v>88.45687552600226</v>
+        <v>88.45687552600209</v>
       </c>
       <c r="I6" t="n">
-        <v>52.12055730830104</v>
+        <v>52.12055730830092</v>
       </c>
       <c r="J6" t="n">
-        <v>59.64120545530873</v>
+        <v>59.64120545530871</v>
       </c>
     </row>
     <row r="7">
@@ -655,28 +655,28 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>351.1725861707304</v>
+        <v>351.1725861707307</v>
       </c>
       <c r="D7" t="n">
-        <v>348.6447727954119</v>
+        <v>348.6447727954118</v>
       </c>
       <c r="E7" t="n">
-        <v>180.6883096067594</v>
+        <v>180.6883096067601</v>
       </c>
       <c r="F7" t="n">
-        <v>189.4028291463326</v>
+        <v>189.4028291463325</v>
       </c>
       <c r="G7" t="n">
-        <v>249.9997159843519</v>
+        <v>249.9997159843515</v>
       </c>
       <c r="H7" t="n">
-        <v>253.5396689430342</v>
+        <v>253.5396689430343</v>
       </c>
       <c r="I7" t="n">
         <v>152.1486568188764</v>
       </c>
       <c r="J7" t="n">
-        <v>154.743308489509</v>
+        <v>154.7433084895086</v>
       </c>
     </row>
     <row r="8">
@@ -689,28 +689,28 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>91.21498193464643</v>
+        <v>91.21498193464646</v>
       </c>
       <c r="D8" t="n">
         <v>103.309214333098</v>
       </c>
       <c r="E8" t="n">
-        <v>56.77080629249633</v>
+        <v>56.77080629249637</v>
       </c>
       <c r="F8" t="n">
-        <v>68.79404002400315</v>
+        <v>68.79404002400314</v>
       </c>
       <c r="G8" t="n">
-        <v>78.78261801769274</v>
+        <v>78.78261801769277</v>
       </c>
       <c r="H8" t="n">
-        <v>86.00659049986028</v>
+        <v>86.00659049986024</v>
       </c>
       <c r="I8" t="n">
         <v>51.04280531572221</v>
       </c>
       <c r="J8" t="n">
-        <v>58.50898816575106</v>
+        <v>58.50898816575107</v>
       </c>
     </row>
     <row r="9">
@@ -726,10 +726,10 @@
         <v>5.396777002201504</v>
       </c>
       <c r="D9" t="n">
-        <v>7.238392296605101</v>
+        <v>7.238392296605102</v>
       </c>
       <c r="E9" t="n">
-        <v>4.262454097575374</v>
+        <v>4.262454097575373</v>
       </c>
       <c r="F9" t="n">
         <v>5.462481231194097</v>
@@ -738,7 +738,7 @@
         <v>5.460263310023226</v>
       </c>
       <c r="H9" t="n">
-        <v>6.325144794949649</v>
+        <v>6.325144794949648</v>
       </c>
       <c r="I9" t="n">
         <v>3.430579416079823</v>
@@ -794,10 +794,10 @@
         <v>4.549466793051771</v>
       </c>
       <c r="D11" t="n">
-        <v>5.627613754023952</v>
+        <v>5.627613754023953</v>
       </c>
       <c r="E11" t="n">
-        <v>2.488115533117207</v>
+        <v>2.488115533117208</v>
       </c>
       <c r="F11" t="n">
         <v>4.428723656331918</v>
@@ -806,13 +806,13 @@
         <v>4.693135964918298</v>
       </c>
       <c r="H11" t="n">
-        <v>5.185076946952907</v>
+        <v>5.185076946952906</v>
       </c>
       <c r="I11" t="n">
         <v>2.988792046532703</v>
       </c>
       <c r="J11" t="n">
-        <v>3.906134132838234</v>
+        <v>3.906134132838233</v>
       </c>
     </row>
     <row r="12">
@@ -828,25 +828,25 @@
         <v>25.80531982009284</v>
       </c>
       <c r="D12" t="n">
-        <v>27.94356194349893</v>
+        <v>27.94356194349891</v>
       </c>
       <c r="E12" t="n">
-        <v>13.75880574035962</v>
+        <v>13.75880574035961</v>
       </c>
       <c r="F12" t="n">
         <v>20.27008709396942</v>
       </c>
       <c r="G12" t="n">
-        <v>25.4501351377888</v>
+        <v>25.45013513778881</v>
       </c>
       <c r="H12" t="n">
-        <v>26.09917424877576</v>
+        <v>26.0991742487758</v>
       </c>
       <c r="I12" t="n">
         <v>15.46594732242185</v>
       </c>
       <c r="J12" t="n">
-        <v>16.35658206641338</v>
+        <v>16.35658206641339</v>
       </c>
     </row>
     <row r="13">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2.694903471242468</v>
+        <v>2.694903471242467</v>
       </c>
       <c r="D13" t="n">
         <v>2.798717303225703</v>
@@ -868,13 +868,13 @@
         <v>3.162651779912894</v>
       </c>
       <c r="F13" t="n">
-        <v>4.814166574567277</v>
+        <v>4.814166574567279</v>
       </c>
       <c r="G13" t="n">
         <v>6.000459378047585</v>
       </c>
       <c r="H13" t="n">
-        <v>5.993342757877886</v>
+        <v>5.993342757877887</v>
       </c>
       <c r="I13" t="n">
         <v>3.653260526487566</v>
@@ -899,22 +899,22 @@
         <v>11.67598164242878</v>
       </c>
       <c r="E14" t="n">
-        <v>7.050096453902311</v>
+        <v>7.050096453902313</v>
       </c>
       <c r="F14" t="n">
-        <v>7.746359461828579</v>
+        <v>7.74635946182858</v>
       </c>
       <c r="G14" t="n">
-        <v>9.221978581692126</v>
+        <v>9.221978581692122</v>
       </c>
       <c r="H14" t="n">
-        <v>9.71675115791655</v>
+        <v>9.716751157916553</v>
       </c>
       <c r="I14" t="n">
         <v>6.004224257755155</v>
       </c>
       <c r="J14" t="n">
-        <v>6.566983138705326</v>
+        <v>6.566983138705323</v>
       </c>
     </row>
     <row r="15">
@@ -930,7 +930,7 @@
         <v>2.318458301455293</v>
       </c>
       <c r="D15" t="n">
-        <v>2.62741115517316</v>
+        <v>2.627411155173159</v>
       </c>
       <c r="E15" t="n">
         <v>1.053014907369696</v>
@@ -945,7 +945,7 @@
         <v>1.382702510500624</v>
       </c>
       <c r="I15" t="n">
-        <v>0.8812554679020421</v>
+        <v>0.8812554679020425</v>
       </c>
       <c r="J15" t="n">
         <v>0.9297606829696782</v>
@@ -961,22 +961,22 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>5.111690432509001</v>
+        <v>5.111690432509</v>
       </c>
       <c r="D16" t="n">
-        <v>5.771543697981107</v>
+        <v>5.771543697981106</v>
       </c>
       <c r="E16" t="n">
-        <v>2.689893464901938</v>
+        <v>2.68989346490194</v>
       </c>
       <c r="F16" t="n">
-        <v>4.22563394595246</v>
+        <v>4.225633945952461</v>
       </c>
       <c r="G16" t="n">
-        <v>5.530143829470427</v>
+        <v>5.53014382947043</v>
       </c>
       <c r="H16" t="n">
-        <v>5.423522195130398</v>
+        <v>5.423522195130396</v>
       </c>
       <c r="I16" t="n">
         <v>3.225212939069747</v>
@@ -995,28 +995,28 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1.704471553824379</v>
+        <v>1.461154248912353</v>
       </c>
       <c r="D17" t="n">
-        <v>1.956188282824467</v>
+        <v>1.701215266220139</v>
       </c>
       <c r="E17" t="n">
-        <v>2.749902009899179</v>
+        <v>0.7328620788712455</v>
       </c>
       <c r="F17" t="n">
-        <v>4.391759273360954</v>
+        <v>1.085113415622173</v>
       </c>
       <c r="G17" t="n">
-        <v>5.152442545354864</v>
+        <v>1.340530232425145</v>
       </c>
       <c r="H17" t="n">
-        <v>5.231266005087943</v>
+        <v>1.407417828345132</v>
       </c>
       <c r="I17" t="n">
-        <v>3.260205307586195</v>
+        <v>0.8344338083239502</v>
       </c>
       <c r="J17" t="n">
-        <v>3.405441380386142</v>
+        <v>0.8769197674874256</v>
       </c>
     </row>
     <row r="18">
@@ -1032,16 +1032,16 @@
         <v>3.669105219633969</v>
       </c>
       <c r="D18" t="n">
-        <v>4.282714717202243</v>
+        <v>4.282714717202245</v>
       </c>
       <c r="E18" t="n">
         <v>1.753700440016704</v>
       </c>
       <c r="F18" t="n">
-        <v>2.830408522286285</v>
+        <v>2.830408522286286</v>
       </c>
       <c r="G18" t="n">
-        <v>3.714936378285149</v>
+        <v>3.714936378285148</v>
       </c>
       <c r="H18" t="n">
         <v>3.773415342782011</v>
@@ -1063,10 +1063,10 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2.748822055575936</v>
+        <v>2.748822055575937</v>
       </c>
       <c r="D19" t="n">
-        <v>3.121114495834338</v>
+        <v>3.121114495834339</v>
       </c>
       <c r="E19" t="n">
         <v>1.612303953812515</v>
@@ -1078,10 +1078,10 @@
         <v>2.662930892094227</v>
       </c>
       <c r="H19" t="n">
-        <v>2.857288834027122</v>
+        <v>2.857288834027121</v>
       </c>
       <c r="I19" t="n">
-        <v>1.668989888367328</v>
+        <v>1.668989888367329</v>
       </c>
       <c r="J19" t="n">
         <v>1.910706642341305</v>
@@ -1097,25 +1097,25 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>9.699166749269562</v>
+        <v>9.699166749269557</v>
       </c>
       <c r="D20" t="n">
-        <v>12.65526906612887</v>
+        <v>12.65526906612888</v>
       </c>
       <c r="E20" t="n">
-        <v>4.82280606925918</v>
+        <v>4.822806069259176</v>
       </c>
       <c r="F20" t="n">
-        <v>8.101692745074356</v>
+        <v>8.101692745074352</v>
       </c>
       <c r="G20" t="n">
         <v>10.05366456704767</v>
       </c>
       <c r="H20" t="n">
-        <v>10.82750015206569</v>
+        <v>10.8275001520657</v>
       </c>
       <c r="I20" t="n">
-        <v>5.765613592184129</v>
+        <v>5.76561359218413</v>
       </c>
       <c r="J20" t="n">
         <v>6.430585764625243</v>
@@ -1168,19 +1168,19 @@
         <v>0.7206993458156795</v>
       </c>
       <c r="D22" t="n">
-        <v>0.7899009717615112</v>
+        <v>0.7899009717615114</v>
       </c>
       <c r="E22" t="n">
-        <v>0.4092245844227267</v>
+        <v>0.4092245844227268</v>
       </c>
       <c r="F22" t="n">
-        <v>0.5959439655928983</v>
+        <v>0.5959439655928984</v>
       </c>
       <c r="G22" t="n">
-        <v>0.7432721765816969</v>
+        <v>0.7432721765816971</v>
       </c>
       <c r="H22" t="n">
-        <v>0.7632870286434741</v>
+        <v>0.7632870286434739</v>
       </c>
       <c r="I22" t="n">
         <v>0.4630559366585686</v>
@@ -1199,10 +1199,10 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>6.504884631329307</v>
+        <v>6.504884631329306</v>
       </c>
       <c r="D23" t="n">
-        <v>6.830307083783942</v>
+        <v>6.830307083783941</v>
       </c>
       <c r="E23" t="n">
         <v>3.547417665170137</v>
@@ -1211,16 +1211,16 @@
         <v>4.176643467945262</v>
       </c>
       <c r="G23" t="n">
-        <v>4.965512237046597</v>
+        <v>4.965512237046598</v>
       </c>
       <c r="H23" t="n">
         <v>5.050810848814081</v>
       </c>
       <c r="I23" t="n">
-        <v>3.242101155092457</v>
+        <v>3.242101155092458</v>
       </c>
       <c r="J23" t="n">
-        <v>3.483772913684959</v>
+        <v>3.48377291368496</v>
       </c>
     </row>
     <row r="24">
@@ -1242,19 +1242,19 @@
         <v>0.04144622646087479</v>
       </c>
       <c r="F24" t="n">
-        <v>0.08246578346383493</v>
+        <v>0.08246578346383492</v>
       </c>
       <c r="G24" t="n">
         <v>0.1097303288847865</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1124322246407573</v>
+        <v>0.1124322246407572</v>
       </c>
       <c r="I24" t="n">
         <v>0.06277715770081188</v>
       </c>
       <c r="J24" t="n">
-        <v>0.06447201611397201</v>
+        <v>0.06447201611397198</v>
       </c>
     </row>
     <row r="25">
@@ -1267,10 +1267,10 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1.507975564067383</v>
+        <v>1.507975564067382</v>
       </c>
       <c r="D25" t="n">
-        <v>1.696747996178411</v>
+        <v>1.69674799617841</v>
       </c>
       <c r="E25" t="n">
         <v>1.104871509412168</v>
@@ -1282,13 +1282,13 @@
         <v>1.370846591996518</v>
       </c>
       <c r="H25" t="n">
-        <v>1.467054385425054</v>
+        <v>1.467054385425055</v>
       </c>
       <c r="I25" t="n">
         <v>0.821444817746862</v>
       </c>
       <c r="J25" t="n">
-        <v>0.9536179656925176</v>
+        <v>0.9536179656925177</v>
       </c>
     </row>
     <row r="26">
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2.935272773140177</v>
+        <v>2.935272773140176</v>
       </c>
       <c r="D26" t="n">
         <v>3.348393162865471</v>
@@ -1313,16 +1313,16 @@
         <v>2.076321378033569</v>
       </c>
       <c r="G26" t="n">
-        <v>2.906452513983364</v>
+        <v>2.906452513983365</v>
       </c>
       <c r="H26" t="n">
-        <v>2.893924685173482</v>
+        <v>2.893924685173481</v>
       </c>
       <c r="I26" t="n">
         <v>1.672702815767416</v>
       </c>
       <c r="J26" t="n">
-        <v>1.741944039571711</v>
+        <v>1.74194403957171</v>
       </c>
     </row>
     <row r="27">
@@ -1338,25 +1338,25 @@
         <v>12.86312213414026</v>
       </c>
       <c r="D27" t="n">
-        <v>12.946331312041</v>
+        <v>12.94633131204099</v>
       </c>
       <c r="E27" t="n">
         <v>8.023853174412972</v>
       </c>
       <c r="F27" t="n">
-        <v>7.048748302135475</v>
+        <v>7.048748302135476</v>
       </c>
       <c r="G27" t="n">
-        <v>8.858010613598637</v>
+        <v>8.858010613598639</v>
       </c>
       <c r="H27" t="n">
-        <v>9.823058512047604</v>
+        <v>9.823058512047607</v>
       </c>
       <c r="I27" t="n">
-        <v>5.902580928679582</v>
+        <v>5.902580928679583</v>
       </c>
       <c r="J27" t="n">
-        <v>5.398246633521766</v>
+        <v>5.398246633521762</v>
       </c>
     </row>
     <row r="28">
@@ -1369,16 +1369,16 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.591618488914628</v>
+        <v>0.5916184889146276</v>
       </c>
       <c r="D28" t="n">
-        <v>0.6663352937639049</v>
+        <v>0.6663352937639045</v>
       </c>
       <c r="E28" t="n">
-        <v>0.2849609254474353</v>
+        <v>0.2849609254474352</v>
       </c>
       <c r="F28" t="n">
-        <v>0.4598894277358185</v>
+        <v>0.4598894277358184</v>
       </c>
       <c r="G28" t="n">
         <v>0.5572436060846812</v>
@@ -1387,10 +1387,10 @@
         <v>0.5976083642872891</v>
       </c>
       <c r="I28" t="n">
-        <v>0.3630871263092579</v>
+        <v>0.3630871263092578</v>
       </c>
       <c r="J28" t="n">
-        <v>0.366884180365224</v>
+        <v>0.3668841803652239</v>
       </c>
     </row>
     <row r="29">
@@ -1403,28 +1403,28 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>17.39931836692441</v>
+        <v>17.39931836692442</v>
       </c>
       <c r="D29" t="n">
-        <v>19.07889196687848</v>
+        <v>19.07889196687847</v>
       </c>
       <c r="E29" t="n">
         <v>14.75064279896196</v>
       </c>
       <c r="F29" t="n">
-        <v>22.9679107342616</v>
+        <v>22.96791073426161</v>
       </c>
       <c r="G29" t="n">
         <v>31.6188788318716</v>
       </c>
       <c r="H29" t="n">
-        <v>28.94252950879505</v>
+        <v>28.94252950879504</v>
       </c>
       <c r="I29" t="n">
-        <v>17.94902666938066</v>
+        <v>17.94902666938067</v>
       </c>
       <c r="J29" t="n">
-        <v>18.74920646793549</v>
+        <v>18.7492064679355</v>
       </c>
     </row>
     <row r="30">
@@ -1440,13 +1440,13 @@
         <v>0.03946551697118005</v>
       </c>
       <c r="D30" t="n">
-        <v>0.04345231628656022</v>
+        <v>0.04345231628656021</v>
       </c>
       <c r="E30" t="n">
         <v>0.01833745408592528</v>
       </c>
       <c r="F30" t="n">
-        <v>0.02405302651294435</v>
+        <v>0.02405302651294436</v>
       </c>
       <c r="G30" t="n">
         <v>0.03307479242791971</v>
@@ -1489,10 +1489,10 @@
         <v>0.01403704581210361</v>
       </c>
       <c r="I31" t="n">
-        <v>0.008379725375248588</v>
+        <v>0.00837972537524859</v>
       </c>
       <c r="J31" t="n">
-        <v>0.007847109271937722</v>
+        <v>0.007847109271937724</v>
       </c>
     </row>
     <row r="32">
@@ -1505,7 +1505,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>26.6642520768732</v>
+        <v>26.66425207687321</v>
       </c>
       <c r="D32" t="n">
         <v>29.04270595907331</v>
@@ -1514,13 +1514,13 @@
         <v>12.66490295939646</v>
       </c>
       <c r="F32" t="n">
-        <v>16.92976931739004</v>
+        <v>16.92976931739003</v>
       </c>
       <c r="G32" t="n">
-        <v>22.21841836935659</v>
+        <v>22.21841836935658</v>
       </c>
       <c r="H32" t="n">
-        <v>23.6353324815287</v>
+        <v>23.63533248152869</v>
       </c>
       <c r="I32" t="n">
         <v>13.58169712299393</v>
@@ -1542,19 +1542,19 @@
         <v>15.47662572463646</v>
       </c>
       <c r="D33" t="n">
-        <v>15.78125430203538</v>
+        <v>15.78125430203537</v>
       </c>
       <c r="E33" t="n">
-        <v>12.10390173394598</v>
+        <v>12.10390173394599</v>
       </c>
       <c r="F33" t="n">
-        <v>14.76305668573948</v>
+        <v>14.76305668573947</v>
       </c>
       <c r="G33" t="n">
         <v>15.38372698370426</v>
       </c>
       <c r="H33" t="n">
-        <v>16.86159724858117</v>
+        <v>16.86159724858116</v>
       </c>
       <c r="I33" t="n">
         <v>10.02759744558886</v>
@@ -1579,10 +1579,10 @@
         <v>1.380940044726551</v>
       </c>
       <c r="E34" t="n">
-        <v>0.6846310907406705</v>
+        <v>0.6846310907406704</v>
       </c>
       <c r="F34" t="n">
-        <v>0.9857493986068436</v>
+        <v>0.9857493986068435</v>
       </c>
       <c r="G34" t="n">
         <v>1.091024202112491</v>
@@ -1591,10 +1591,10 @@
         <v>1.20153631061961</v>
       </c>
       <c r="I34" t="n">
-        <v>0.7400941028300339</v>
+        <v>0.7400941028300336</v>
       </c>
       <c r="J34" t="n">
-        <v>0.8146899753003479</v>
+        <v>0.8146899753003478</v>
       </c>
     </row>
     <row r="35">
@@ -1607,7 +1607,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0.5030096675405571</v>
+        <v>0.5030096675405572</v>
       </c>
       <c r="D35" t="n">
         <v>0.5200546352624036</v>
@@ -1616,7 +1616,7 @@
         <v>0.4260941926272812</v>
       </c>
       <c r="F35" t="n">
-        <v>0.4602144274222585</v>
+        <v>0.4602144274222586</v>
       </c>
       <c r="G35" t="n">
         <v>0.4743810580795903</v>
@@ -1647,7 +1647,7 @@
         <v>1.874595946852974</v>
       </c>
       <c r="E36" t="n">
-        <v>0.7621406334507139</v>
+        <v>0.7621406334507138</v>
       </c>
       <c r="F36" t="n">
         <v>1.176563179133914</v>
@@ -1662,7 +1662,7 @@
         <v>0.9073022773706648</v>
       </c>
       <c r="J36" t="n">
-        <v>0.9344442427404437</v>
+        <v>0.9344442427404438</v>
       </c>
     </row>
     <row r="37">
@@ -1681,7 +1681,7 @@
         <v>12.76301483027557</v>
       </c>
       <c r="E37" t="n">
-        <v>6.251050519830937</v>
+        <v>6.251050519830939</v>
       </c>
       <c r="F37" t="n">
         <v>6.710316511361758</v>
@@ -1709,7 +1709,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0.7849469160883628</v>
+        <v>0.7849469160883626</v>
       </c>
       <c r="D38" t="n">
         <v>0.9132989918408624</v>
@@ -1718,10 +1718,10 @@
         <v>0.3258197497202404</v>
       </c>
       <c r="F38" t="n">
-        <v>0.5369941155911732</v>
+        <v>0.5369941155911733</v>
       </c>
       <c r="G38" t="n">
-        <v>0.6994609993106571</v>
+        <v>0.6994609993106569</v>
       </c>
       <c r="H38" t="n">
         <v>0.7111237469169237</v>
@@ -1777,7 +1777,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0.09137906212440466</v>
+        <v>0.09137906212440465</v>
       </c>
       <c r="D40" t="n">
         <v>0.114431119821943</v>
@@ -1792,7 +1792,7 @@
         <v>0.09788196374805611</v>
       </c>
       <c r="H40" t="n">
-        <v>0.1124300560865089</v>
+        <v>0.112430056086509</v>
       </c>
       <c r="I40" t="n">
         <v>0.06217414423843794</v>
@@ -1811,13 +1811,13 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>0.5756599885946353</v>
+        <v>0.5756599885946351</v>
       </c>
       <c r="D41" t="n">
         <v>0.6832611117792142</v>
       </c>
       <c r="E41" t="n">
-        <v>0.4290283019552805</v>
+        <v>0.4290283019552806</v>
       </c>
       <c r="F41" t="n">
         <v>0.5710133063068424</v>
@@ -1826,13 +1826,13 @@
         <v>0.6159109831792959</v>
       </c>
       <c r="H41" t="n">
-        <v>0.6500139003678751</v>
+        <v>0.6500139003678752</v>
       </c>
       <c r="I41" t="n">
         <v>0.3786361406106325</v>
       </c>
       <c r="J41" t="n">
-        <v>0.4568192666566003</v>
+        <v>0.4568192666566002</v>
       </c>
     </row>
     <row r="42">
@@ -1851,22 +1851,22 @@
         <v>0.6902305357084338</v>
       </c>
       <c r="E42" t="n">
-        <v>0.4131685613799904</v>
+        <v>0.4131685613799903</v>
       </c>
       <c r="F42" t="n">
-        <v>0.5401845995576061</v>
+        <v>0.5401845995576062</v>
       </c>
       <c r="G42" t="n">
         <v>0.5886096716663801</v>
       </c>
       <c r="H42" t="n">
-        <v>0.6189795265900536</v>
+        <v>0.6189795265900538</v>
       </c>
       <c r="I42" t="n">
         <v>0.3740987448795141</v>
       </c>
       <c r="J42" t="n">
-        <v>0.4282451340990709</v>
+        <v>0.4282451340990711</v>
       </c>
     </row>
     <row r="43">
@@ -1879,7 +1879,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1.539860423727769</v>
+        <v>1.539860423727768</v>
       </c>
       <c r="D43" t="n">
         <v>1.748445481633528</v>
@@ -1888,7 +1888,7 @@
         <v>1.593202202599534</v>
       </c>
       <c r="F43" t="n">
-        <v>1.627214438307768</v>
+        <v>1.627214438307769</v>
       </c>
       <c r="G43" t="n">
         <v>1.441744142717568</v>
@@ -1897,7 +1897,7 @@
         <v>1.801237855415094</v>
       </c>
       <c r="I43" t="n">
-        <v>0.9975328080110334</v>
+        <v>0.9975328080110333</v>
       </c>
       <c r="J43" t="n">
         <v>1.391823077789894</v>
@@ -1919,19 +1919,19 @@
         <v>4.041392324023093</v>
       </c>
       <c r="E44" t="n">
-        <v>2.095404661669109</v>
+        <v>2.09540466166911</v>
       </c>
       <c r="F44" t="n">
-        <v>2.692782209011392</v>
+        <v>2.692782209011391</v>
       </c>
       <c r="G44" t="n">
-        <v>3.400334089286146</v>
+        <v>3.400334089286148</v>
       </c>
       <c r="H44" t="n">
         <v>3.583375402353514</v>
       </c>
       <c r="I44" t="n">
-        <v>2.114546101550435</v>
+        <v>2.114546101550437</v>
       </c>
       <c r="J44" t="n">
         <v>2.14766310345164</v>
@@ -1984,10 +1984,10 @@
         <v>0.1498766047835814</v>
       </c>
       <c r="D46" t="n">
-        <v>0.1650543105975262</v>
+        <v>0.1650543105975263</v>
       </c>
       <c r="E46" t="n">
-        <v>0.08964448593307885</v>
+        <v>0.08964448593307886</v>
       </c>
       <c r="F46" t="n">
         <v>0.1497160452346641</v>
@@ -1999,7 +1999,7 @@
         <v>0.1674936501473765</v>
       </c>
       <c r="I46" t="n">
-        <v>0.1007983391337059</v>
+        <v>0.100798339133706</v>
       </c>
       <c r="J46" t="n">
         <v>0.1277258451288606</v>
@@ -2052,25 +2052,25 @@
         <v>1.382782313131683</v>
       </c>
       <c r="D48" t="n">
-        <v>1.513366896511472</v>
+        <v>1.513366896511471</v>
       </c>
       <c r="E48" t="n">
         <v>0.627259571177382</v>
       </c>
       <c r="F48" t="n">
-        <v>1.023363371543038</v>
+        <v>1.023363371543039</v>
       </c>
       <c r="G48" t="n">
-        <v>0.927557934994753</v>
+        <v>0.9275579349947529</v>
       </c>
       <c r="H48" t="n">
         <v>1.065718509364393</v>
       </c>
       <c r="I48" t="n">
-        <v>0.6189859122012801</v>
+        <v>0.6189859122012802</v>
       </c>
       <c r="J48" t="n">
-        <v>0.9778741378348969</v>
+        <v>0.9778741378348965</v>
       </c>
     </row>
     <row r="49">
@@ -2101,7 +2101,7 @@
         <v>15.76535108785712</v>
       </c>
       <c r="I49" t="n">
-        <v>9.952180216568678</v>
+        <v>9.952180216568676</v>
       </c>
       <c r="J49" t="n">
         <v>8.867717797858994</v>
@@ -2117,25 +2117,25 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>0.8703737401465719</v>
+        <v>0.8703737401465717</v>
       </c>
       <c r="D50" t="n">
         <v>0.8646103157382035</v>
       </c>
       <c r="E50" t="n">
-        <v>0.3335112776995508</v>
+        <v>0.3335112776995509</v>
       </c>
       <c r="F50" t="n">
-        <v>0.3778265802658275</v>
+        <v>0.3778265802658274</v>
       </c>
       <c r="G50" t="n">
         <v>0.5235500107591835</v>
       </c>
       <c r="H50" t="n">
-        <v>0.5326108726426459</v>
+        <v>0.5326108726426458</v>
       </c>
       <c r="I50" t="n">
-        <v>0.3016761224771969</v>
+        <v>0.301676122477197</v>
       </c>
       <c r="J50" t="n">
         <v>0.2918915195470023</v>
@@ -2151,10 +2151,10 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>38.60826127613986</v>
+        <v>38.60826127613985</v>
       </c>
       <c r="D51" t="n">
-        <v>39.23658226310143</v>
+        <v>39.2365822631014</v>
       </c>
       <c r="E51" t="n">
         <v>18.32370669359452</v>
@@ -2185,10 +2185,10 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>0.28337951025255</v>
+        <v>0.2833795102525499</v>
       </c>
       <c r="D52" t="n">
-        <v>0.3061723668201927</v>
+        <v>0.3061723668201928</v>
       </c>
       <c r="E52" t="n">
         <v>0.2199678091310042</v>
@@ -2206,7 +2206,7 @@
         <v>0.2232603731717787</v>
       </c>
       <c r="J52" t="n">
-        <v>0.2113398403110085</v>
+        <v>0.2113398403110084</v>
       </c>
     </row>
     <row r="53">
@@ -2219,28 +2219,28 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0.1587525061594246</v>
+        <v>0.1587525061594245</v>
       </c>
       <c r="D53" t="n">
         <v>0.1770817401368001</v>
       </c>
       <c r="E53" t="n">
-        <v>0.07631215799237652</v>
+        <v>0.07631215799237653</v>
       </c>
       <c r="F53" t="n">
         <v>0.1088267567256846</v>
       </c>
       <c r="G53" t="n">
-        <v>0.1470830715245102</v>
+        <v>0.1470830715245101</v>
       </c>
       <c r="H53" t="n">
         <v>0.1424796353226244</v>
       </c>
       <c r="I53" t="n">
-        <v>0.08252963741466346</v>
+        <v>0.08252963741466345</v>
       </c>
       <c r="J53" t="n">
-        <v>0.0832265156639885</v>
+        <v>0.08322651566398852</v>
       </c>
     </row>
     <row r="54">
@@ -2262,13 +2262,13 @@
         <v>11.09473282335949</v>
       </c>
       <c r="F54" t="n">
-        <v>16.55762423110096</v>
+        <v>16.55762423110097</v>
       </c>
       <c r="G54" t="n">
         <v>16.39074970450189</v>
       </c>
       <c r="H54" t="n">
-        <v>18.11194150470611</v>
+        <v>18.1119415047061</v>
       </c>
       <c r="I54" t="n">
         <v>11.08726278481308</v>
@@ -2287,28 +2287,28 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>4.837869476991521</v>
+        <v>4.837869476991523</v>
       </c>
       <c r="D55" t="n">
-        <v>5.683982241098268</v>
+        <v>5.68398224109827</v>
       </c>
       <c r="E55" t="n">
-        <v>3.509544806186098</v>
+        <v>3.509544806186099</v>
       </c>
       <c r="F55" t="n">
-        <v>4.867686430737443</v>
+        <v>4.867686430737442</v>
       </c>
       <c r="G55" t="n">
-        <v>4.640737621381624</v>
+        <v>4.640737621381625</v>
       </c>
       <c r="H55" t="n">
-        <v>5.332243900948134</v>
+        <v>5.332243900948135</v>
       </c>
       <c r="I55" t="n">
         <v>3.110861467339314</v>
       </c>
       <c r="J55" t="n">
-        <v>3.780553353471421</v>
+        <v>3.78055335347142</v>
       </c>
     </row>
     <row r="56">
@@ -2327,19 +2327,19 @@
         <v>12.38629341870544</v>
       </c>
       <c r="E56" t="n">
-        <v>4.505496183044798</v>
+        <v>4.505496183044797</v>
       </c>
       <c r="F56" t="n">
-        <v>4.937833246191836</v>
+        <v>4.937833246191837</v>
       </c>
       <c r="G56" t="n">
-        <v>9.445351730424248</v>
+        <v>9.445351730424242</v>
       </c>
       <c r="H56" t="n">
-        <v>9.566128422368875</v>
+        <v>9.566128422368877</v>
       </c>
       <c r="I56" t="n">
-        <v>4.420091163675151</v>
+        <v>4.420091163675152</v>
       </c>
       <c r="J56" t="n">
         <v>4.700991802924555</v>
@@ -2358,16 +2358,16 @@
         <v>0.7144709180789534</v>
       </c>
       <c r="D57" t="n">
-        <v>0.8372439121545082</v>
+        <v>0.8372439121545083</v>
       </c>
       <c r="E57" t="n">
-        <v>0.4329023545836814</v>
+        <v>0.4329023545836813</v>
       </c>
       <c r="F57" t="n">
-        <v>0.617341974264683</v>
+        <v>0.6173419742646828</v>
       </c>
       <c r="G57" t="n">
-        <v>0.6493436670692699</v>
+        <v>0.6493436670692698</v>
       </c>
       <c r="H57" t="n">
         <v>0.705658238573004</v>
@@ -2389,25 +2389,25 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>0.7802397160530992</v>
+        <v>0.7802397160530991</v>
       </c>
       <c r="D58" t="n">
-        <v>0.887813688223257</v>
+        <v>0.8878136882232575</v>
       </c>
       <c r="E58" t="n">
         <v>0.3703870886852618</v>
       </c>
       <c r="F58" t="n">
-        <v>0.6095971369903236</v>
+        <v>0.6095971369903235</v>
       </c>
       <c r="G58" t="n">
-        <v>0.7106269353447004</v>
+        <v>0.7106269353447003</v>
       </c>
       <c r="H58" t="n">
         <v>0.7413372762098162</v>
       </c>
       <c r="I58" t="n">
-        <v>0.3865546352852068</v>
+        <v>0.3865546352852067</v>
       </c>
       <c r="J58" t="n">
         <v>0.5171024930467497</v>
@@ -2429,22 +2429,22 @@
         <v>1.123948365378146</v>
       </c>
       <c r="E59" t="n">
-        <v>0.5303691467818078</v>
+        <v>0.5303691467818077</v>
       </c>
       <c r="F59" t="n">
-        <v>0.6451331484040023</v>
+        <v>0.645133148404002</v>
       </c>
       <c r="G59" t="n">
-        <v>0.8528120210492669</v>
+        <v>0.8528120210492667</v>
       </c>
       <c r="H59" t="n">
-        <v>0.88655877555773</v>
+        <v>0.8865587755577297</v>
       </c>
       <c r="I59" t="n">
-        <v>0.504095619571324</v>
+        <v>0.5040956195713239</v>
       </c>
       <c r="J59" t="n">
-        <v>0.5246744291473068</v>
+        <v>0.5246744291473071</v>
       </c>
     </row>
     <row r="60">
@@ -2457,7 +2457,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>3.725572610146813</v>
+        <v>3.725572610146814</v>
       </c>
       <c r="D60" t="n">
         <v>3.687439615258409</v>
@@ -2469,16 +2469,16 @@
         <v>3.57093062303586</v>
       </c>
       <c r="G60" t="n">
-        <v>4.619149193672878</v>
+        <v>4.61914919367288</v>
       </c>
       <c r="H60" t="n">
         <v>4.50990368540872</v>
       </c>
       <c r="I60" t="n">
-        <v>2.853681654067374</v>
+        <v>2.853681654067373</v>
       </c>
       <c r="J60" t="n">
-        <v>2.88026763327106</v>
+        <v>2.880267633271061</v>
       </c>
     </row>
     <row r="61">
@@ -2494,7 +2494,7 @@
         <v>0.207576457682</v>
       </c>
       <c r="D61" t="n">
-        <v>0.2435677918138836</v>
+        <v>0.2435677918138837</v>
       </c>
       <c r="E61" t="n">
         <v>0.1706830883634576</v>
@@ -2509,10 +2509,10 @@
         <v>0.3107919444184356</v>
       </c>
       <c r="I61" t="n">
-        <v>0.2007706186907537</v>
+        <v>0.2007706186907536</v>
       </c>
       <c r="J61" t="n">
-        <v>0.2289922216844853</v>
+        <v>0.2289922216844852</v>
       </c>
     </row>
     <row r="62">
@@ -2528,7 +2528,7 @@
         <v>0.5863970507192008</v>
       </c>
       <c r="D62" t="n">
-        <v>0.5570501220765453</v>
+        <v>0.5570501220765451</v>
       </c>
       <c r="E62" t="n">
         <v>0.23385395205274</v>
@@ -2574,13 +2574,13 @@
         <v>4.265171395480166</v>
       </c>
       <c r="H63" t="n">
-        <v>4.032080763577189</v>
+        <v>4.03208076357719</v>
       </c>
       <c r="I63" t="n">
         <v>2.545807713626816</v>
       </c>
       <c r="J63" t="n">
-        <v>2.904921084266627</v>
+        <v>2.904921084266626</v>
       </c>
     </row>
     <row r="64">
@@ -2596,7 +2596,7 @@
         <v>0.07910738921069307</v>
       </c>
       <c r="D64" t="n">
-        <v>0.08481796400129639</v>
+        <v>0.0848179640012964</v>
       </c>
       <c r="E64" t="n">
         <v>0.06997316935660622</v>
@@ -2605,10 +2605,10 @@
         <v>0.0820670197056325</v>
       </c>
       <c r="G64" t="n">
-        <v>0.07624540218838934</v>
+        <v>0.07624540218838935</v>
       </c>
       <c r="H64" t="n">
-        <v>0.09109144277065336</v>
+        <v>0.09109144277065334</v>
       </c>
       <c r="I64" t="n">
         <v>0.04948734912003784</v>
@@ -2642,10 +2642,10 @@
         <v>14.37407919848759</v>
       </c>
       <c r="H65" t="n">
-        <v>14.54208313817992</v>
+        <v>14.54208313817991</v>
       </c>
       <c r="I65" t="n">
-        <v>7.938661301698586</v>
+        <v>7.938661301698587</v>
       </c>
       <c r="J65" t="n">
         <v>8.184344886349287</v>
@@ -2670,13 +2670,13 @@
         <v>0.577902642655298</v>
       </c>
       <c r="F66" t="n">
-        <v>0.8592826001497798</v>
+        <v>0.8592826001497799</v>
       </c>
       <c r="G66" t="n">
         <v>0.9981246993290327</v>
       </c>
       <c r="H66" t="n">
-        <v>1.051479126105705</v>
+        <v>1.051479126105704</v>
       </c>
       <c r="I66" t="n">
         <v>0.5956081547720092</v>
@@ -2698,7 +2698,7 @@
         <v>0.03637696884939718</v>
       </c>
       <c r="D67" t="n">
-        <v>0.03861541827141312</v>
+        <v>0.03861541827141311</v>
       </c>
       <c r="E67" t="n">
         <v>0.03216154213516775</v>
@@ -2707,7 +2707,7 @@
         <v>0.03565382322638939</v>
       </c>
       <c r="G67" t="n">
-        <v>0.04195789064130711</v>
+        <v>0.0419578906413071</v>
       </c>
       <c r="H67" t="n">
         <v>0.04186114549071578</v>
@@ -2732,7 +2732,7 @@
         <v>0.2237010692046989</v>
       </c>
       <c r="D68" t="n">
-        <v>0.2538165204273506</v>
+        <v>0.2538165204273507</v>
       </c>
       <c r="E68" t="n">
         <v>0.1669073948016405</v>
@@ -2741,16 +2741,16 @@
         <v>0.2120944157926978</v>
       </c>
       <c r="G68" t="n">
-        <v>0.241523469395261</v>
+        <v>0.2415234693952611</v>
       </c>
       <c r="H68" t="n">
         <v>0.2576083374932814</v>
       </c>
       <c r="I68" t="n">
-        <v>0.1564559625132826</v>
+        <v>0.1564559625132825</v>
       </c>
       <c r="J68" t="n">
-        <v>0.1638314495766678</v>
+        <v>0.1638314495766679</v>
       </c>
     </row>
     <row r="69">
@@ -2766,7 +2766,7 @@
         <v>0.2997928011395921</v>
       </c>
       <c r="D69" t="n">
-        <v>0.305896646570271</v>
+        <v>0.3058966465702709</v>
       </c>
       <c r="E69" t="n">
         <v>0.254457270715416</v>
@@ -2781,7 +2781,7 @@
         <v>0.3544438973644519</v>
       </c>
       <c r="I69" t="n">
-        <v>0.2361565900012201</v>
+        <v>0.23615659000122</v>
       </c>
       <c r="J69" t="n">
         <v>0.2370386651133713</v>
@@ -2831,28 +2831,28 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>5.221240320629952</v>
+        <v>5.22124032062995</v>
       </c>
       <c r="D71" t="n">
-        <v>5.042501633076734</v>
+        <v>5.042501633076735</v>
       </c>
       <c r="E71" t="n">
         <v>5.26852841933967</v>
       </c>
       <c r="F71" t="n">
-        <v>4.850997286526085</v>
+        <v>4.850997286526084</v>
       </c>
       <c r="G71" t="n">
         <v>5.926440538855653</v>
       </c>
       <c r="H71" t="n">
-        <v>5.673522753735333</v>
+        <v>5.673522753735332</v>
       </c>
       <c r="I71" t="n">
         <v>3.63711143996666</v>
       </c>
       <c r="J71" t="n">
-        <v>4.122721220342225</v>
+        <v>4.122721220342224</v>
       </c>
     </row>
     <row r="72">
@@ -2877,7 +2877,7 @@
         <v>1.927498433077062</v>
       </c>
       <c r="G72" t="n">
-        <v>2.57327690592926</v>
+        <v>2.573276905929261</v>
       </c>
       <c r="H72" t="n">
         <v>2.918983310487115</v>
@@ -2899,28 +2899,28 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>3.016643294575578</v>
+        <v>3.016643294575577</v>
       </c>
       <c r="D73" t="n">
-        <v>3.436733153505116</v>
+        <v>3.436733153505115</v>
       </c>
       <c r="E73" t="n">
         <v>1.667411007967831</v>
       </c>
       <c r="F73" t="n">
-        <v>2.044881035307247</v>
+        <v>2.044881035307246</v>
       </c>
       <c r="G73" t="n">
-        <v>2.566589696491706</v>
+        <v>2.566589696491705</v>
       </c>
       <c r="H73" t="n">
-        <v>2.789600531657451</v>
+        <v>2.789600531657449</v>
       </c>
       <c r="I73" t="n">
-        <v>1.610847301674793</v>
+        <v>1.610847301674794</v>
       </c>
       <c r="J73" t="n">
-        <v>1.797558310934366</v>
+        <v>1.797558310934365</v>
       </c>
     </row>
     <row r="74">
@@ -2936,7 +2936,7 @@
         <v>1.972571596661882</v>
       </c>
       <c r="D74" t="n">
-        <v>2.276730638852491</v>
+        <v>2.27673063885249</v>
       </c>
       <c r="E74" t="n">
         <v>1.558919958473936</v>
@@ -3001,7 +3001,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>0.9528720653772792</v>
+        <v>0.9528720653772791</v>
       </c>
       <c r="D76" t="n">
         <v>1.065732962135946</v>
@@ -3010,13 +3010,13 @@
         <v>0.5018812391962425</v>
       </c>
       <c r="F76" t="n">
-        <v>0.6613468117444121</v>
+        <v>0.661346811744412</v>
       </c>
       <c r="G76" t="n">
-        <v>0.8442576078825237</v>
+        <v>0.8442576078825236</v>
       </c>
       <c r="H76" t="n">
-        <v>0.8920308632170663</v>
+        <v>0.8920308632170664</v>
       </c>
       <c r="I76" t="n">
         <v>0.5235427156482182</v>
@@ -3056,7 +3056,7 @@
         <v>0.1777964538598388</v>
       </c>
       <c r="J77" t="n">
-        <v>0.1702877420803483</v>
+        <v>0.1702877420803482</v>
       </c>
     </row>
     <row r="78">
@@ -3109,19 +3109,19 @@
         <v>0.126298568474592</v>
       </c>
       <c r="E79" t="n">
-        <v>0.04187002880907853</v>
+        <v>0.04187002880907852</v>
       </c>
       <c r="F79" t="n">
-        <v>0.07444904272193183</v>
+        <v>0.07444904272193181</v>
       </c>
       <c r="G79" t="n">
-        <v>0.09818708385514124</v>
+        <v>0.09818708385514123</v>
       </c>
       <c r="H79" t="n">
-        <v>0.0995738707421838</v>
+        <v>0.09957387074218381</v>
       </c>
       <c r="I79" t="n">
-        <v>0.05739088347884539</v>
+        <v>0.05739088347884538</v>
       </c>
       <c r="J79" t="n">
         <v>0.06036041992485646</v>
@@ -3146,13 +3146,13 @@
         <v>0.1294624491153893</v>
       </c>
       <c r="F80" t="n">
-        <v>0.1945513364902319</v>
+        <v>0.1945513364902318</v>
       </c>
       <c r="G80" t="n">
         <v>0.1639654104711578</v>
       </c>
       <c r="H80" t="n">
-        <v>0.2140039434831763</v>
+        <v>0.2140039434831764</v>
       </c>
       <c r="I80" t="n">
         <v>0.138662849561895</v>
@@ -3174,25 +3174,25 @@
         <v>0.1183294408639476</v>
       </c>
       <c r="D81" t="n">
-        <v>0.116272743835213</v>
+        <v>0.1162727438352129</v>
       </c>
       <c r="E81" t="n">
         <v>0.07350880577521007</v>
       </c>
       <c r="F81" t="n">
-        <v>0.07022037763293475</v>
+        <v>0.07022037763293473</v>
       </c>
       <c r="G81" t="n">
-        <v>0.08919227449950537</v>
+        <v>0.0891922744995054</v>
       </c>
       <c r="H81" t="n">
         <v>0.09105800781072881</v>
       </c>
       <c r="I81" t="n">
-        <v>0.05693894514937477</v>
+        <v>0.05693894514937478</v>
       </c>
       <c r="J81" t="n">
-        <v>0.05411202299963547</v>
+        <v>0.05411202299963546</v>
       </c>
     </row>
     <row r="82">
@@ -3205,13 +3205,13 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>0.3212667401559587</v>
+        <v>0.3212667401559588</v>
       </c>
       <c r="D82" t="n">
         <v>0.3701078331417929</v>
       </c>
       <c r="E82" t="n">
-        <v>0.117158824664995</v>
+        <v>0.1171588246649949</v>
       </c>
       <c r="F82" t="n">
         <v>0.1520931076018346</v>
@@ -3220,13 +3220,13 @@
         <v>0.2747160548506381</v>
       </c>
       <c r="H82" t="n">
-        <v>0.2761964442231879</v>
+        <v>0.2761964442231878</v>
       </c>
       <c r="I82" t="n">
         <v>0.1353340208157378</v>
       </c>
       <c r="J82" t="n">
-        <v>0.1365448372646572</v>
+        <v>0.1365448372646573</v>
       </c>
     </row>
     <row r="83">
@@ -3273,10 +3273,10 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>0.2811654652006271</v>
+        <v>0.281165465200627</v>
       </c>
       <c r="D84" t="n">
-        <v>0.2932664571408647</v>
+        <v>0.2932664571408646</v>
       </c>
       <c r="E84" t="n">
         <v>0.3830725266129369</v>
@@ -3285,7 +3285,7 @@
         <v>0.3970093234712659</v>
       </c>
       <c r="G84" t="n">
-        <v>0.4212499210414785</v>
+        <v>0.4212499210414786</v>
       </c>
       <c r="H84" t="n">
         <v>0.4846136050582912</v>
@@ -3307,19 +3307,19 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>0.860769933463875</v>
+        <v>0.8607699334638753</v>
       </c>
       <c r="D85" t="n">
-        <v>0.9173134007636821</v>
+        <v>0.917313400763682</v>
       </c>
       <c r="E85" t="n">
-        <v>2.15861916672212</v>
+        <v>2.158619166722119</v>
       </c>
       <c r="F85" t="n">
         <v>3.476123912639208</v>
       </c>
       <c r="G85" t="n">
-        <v>4.126546308813389</v>
+        <v>4.126546308813388</v>
       </c>
       <c r="H85" t="n">
         <v>4.109425649342285</v>
@@ -3328,7 +3328,7 @@
         <v>2.56791451366115</v>
       </c>
       <c r="J85" t="n">
-        <v>2.673025061119595</v>
+        <v>2.673025061119596</v>
       </c>
     </row>
     <row r="86">
@@ -3341,7 +3341,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>0.3667195053327091</v>
+        <v>0.3667195053327092</v>
       </c>
       <c r="D86" t="n">
         <v>0.4229408202713202</v>
@@ -3350,13 +3350,13 @@
         <v>0.2426673331995914</v>
       </c>
       <c r="F86" t="n">
-        <v>0.3445247612395539</v>
+        <v>0.3445247612395538</v>
       </c>
       <c r="G86" t="n">
         <v>0.3917755089857468</v>
       </c>
       <c r="H86" t="n">
-        <v>0.4311755942484279</v>
+        <v>0.431175594248428</v>
       </c>
       <c r="I86" t="n">
         <v>0.27726379153634</v>
@@ -3415,10 +3415,10 @@
         <v>1.339979849185605</v>
       </c>
       <c r="E88" t="n">
-        <v>3.61455936276061</v>
+        <v>3.614559362760611</v>
       </c>
       <c r="F88" t="n">
-        <v>5.856089389219887</v>
+        <v>5.856089389219888</v>
       </c>
       <c r="G88" t="n">
         <v>6.397873875697827</v>
@@ -3427,10 +3427,10 @@
         <v>6.387446047299759</v>
       </c>
       <c r="I88" t="n">
-        <v>4.044828530768766</v>
+        <v>4.044828530768767</v>
       </c>
       <c r="J88" t="n">
-        <v>4.562539980781592</v>
+        <v>4.562539980781593</v>
       </c>
     </row>
     <row r="89">
@@ -3443,7 +3443,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>0.02280443999049884</v>
+        <v>0.02280443999049883</v>
       </c>
       <c r="D89" t="n">
         <v>0.02254113231645363</v>
@@ -3526,7 +3526,7 @@
         <v>0.0433595615979744</v>
       </c>
       <c r="H91" t="n">
-        <v>0.03937700806504067</v>
+        <v>0.03937700806504066</v>
       </c>
       <c r="I91" t="n">
         <v>0.01758838455758589</v>
@@ -3625,10 +3625,10 @@
         <v>0.348780911070835</v>
       </c>
       <c r="G94" t="n">
-        <v>0.5674912128330384</v>
+        <v>0.5674912128330382</v>
       </c>
       <c r="H94" t="n">
-        <v>0.5443135397490282</v>
+        <v>0.5443135397490283</v>
       </c>
       <c r="I94" t="n">
         <v>0.2629254475965794</v>
@@ -3659,10 +3659,10 @@
         <v>0.430009754556704</v>
       </c>
       <c r="G95" t="n">
-        <v>0.8274045788155056</v>
+        <v>0.8274045788155058</v>
       </c>
       <c r="H95" t="n">
-        <v>0.7793599699948628</v>
+        <v>0.7793599699948627</v>
       </c>
       <c r="I95" t="n">
         <v>0.3966146612751346</v>
@@ -3687,7 +3687,7 @@
         <v>0.2788627229166179</v>
       </c>
       <c r="E96" t="n">
-        <v>0.1671774345963504</v>
+        <v>0.1671774345963505</v>
       </c>
       <c r="F96" t="n">
         <v>0.1716992219691555</v>
@@ -3724,19 +3724,19 @@
         <v>0.04911511568663023</v>
       </c>
       <c r="F97" t="n">
-        <v>0.05519384056912498</v>
+        <v>0.05519384056912499</v>
       </c>
       <c r="G97" t="n">
         <v>0.09999335212816846</v>
       </c>
       <c r="H97" t="n">
-        <v>0.09927875045044077</v>
+        <v>0.09927875045044079</v>
       </c>
       <c r="I97" t="n">
         <v>0.05041147983539526</v>
       </c>
       <c r="J97" t="n">
-        <v>0.04787660197334978</v>
+        <v>0.04787660197334979</v>
       </c>
     </row>
     <row r="98">
@@ -3752,7 +3752,7 @@
         <v>0.4101632041115676</v>
       </c>
       <c r="D98" t="n">
-        <v>0.4348800387658589</v>
+        <v>0.4348800387658587</v>
       </c>
       <c r="E98" t="n">
         <v>0.1926547973928941</v>
@@ -3761,16 +3761,16 @@
         <v>0.1980533576898899</v>
       </c>
       <c r="G98" t="n">
-        <v>0.3131421208342071</v>
+        <v>0.3131421208342069</v>
       </c>
       <c r="H98" t="n">
-        <v>0.3113767426089164</v>
+        <v>0.3113767426089163</v>
       </c>
       <c r="I98" t="n">
         <v>0.1714392197989717</v>
       </c>
       <c r="J98" t="n">
-        <v>0.1685549794518724</v>
+        <v>0.1685549794518725</v>
       </c>
     </row>
     <row r="99">
@@ -3820,7 +3820,7 @@
         <v>0.2549202929094538</v>
       </c>
       <c r="D100" t="n">
-        <v>0.2660634751255427</v>
+        <v>0.2660634751255426</v>
       </c>
       <c r="E100" t="n">
         <v>0.1808176225900406</v>
@@ -3829,7 +3829,7 @@
         <v>0.195850303212614</v>
       </c>
       <c r="G100" t="n">
-        <v>0.2226987417056911</v>
+        <v>0.2226987417056912</v>
       </c>
       <c r="H100" t="n">
         <v>0.2379403602734601</v>
@@ -3854,13 +3854,13 @@
         <v>0.2751747646897075</v>
       </c>
       <c r="D101" t="n">
-        <v>0.2952714526551808</v>
+        <v>0.2952714526551809</v>
       </c>
       <c r="E101" t="n">
-        <v>0.09405244592060437</v>
+        <v>0.09405244592060436</v>
       </c>
       <c r="F101" t="n">
-        <v>0.1737979705488479</v>
+        <v>0.173797970548848</v>
       </c>
       <c r="G101" t="n">
         <v>0.238476700088527</v>
@@ -3888,13 +3888,13 @@
         <v>1.798238731243467</v>
       </c>
       <c r="D102" t="n">
-        <v>2.427423946021358</v>
+        <v>2.427423946021357</v>
       </c>
       <c r="E102" t="n">
-        <v>1.319629443472804</v>
+        <v>1.319629443472805</v>
       </c>
       <c r="F102" t="n">
-        <v>1.682614412457483</v>
+        <v>1.682614412457482</v>
       </c>
       <c r="G102" t="n">
         <v>1.786081245807626</v>
@@ -3903,10 +3903,10 @@
         <v>2.073932485035356</v>
       </c>
       <c r="I102" t="n">
-        <v>1.307980667428288</v>
+        <v>1.307980667428287</v>
       </c>
       <c r="J102" t="n">
-        <v>1.393941797215901</v>
+        <v>1.3939417972159</v>
       </c>
     </row>
     <row r="103">
@@ -3928,16 +3928,16 @@
         <v>0.04589006385200817</v>
       </c>
       <c r="F103" t="n">
-        <v>0.06314323250428461</v>
+        <v>0.06314323250428459</v>
       </c>
       <c r="G103" t="n">
         <v>0.09299028313562077</v>
       </c>
       <c r="H103" t="n">
-        <v>0.08902953824928203</v>
+        <v>0.08902953824928204</v>
       </c>
       <c r="I103" t="n">
-        <v>0.05023422101834224</v>
+        <v>0.05023422101834223</v>
       </c>
       <c r="J103" t="n">
         <v>0.05056447810202596</v>
@@ -3965,7 +3965,7 @@
         <v>0.1860963010020512</v>
       </c>
       <c r="G104" t="n">
-        <v>0.2429708744179499</v>
+        <v>0.2429708744179498</v>
       </c>
       <c r="H104" t="n">
         <v>0.2495251606318192</v>
@@ -4042,7 +4042,7 @@
         <v>0.2565968995245774</v>
       </c>
       <c r="J106" t="n">
-        <v>0.2733256079578454</v>
+        <v>0.2733256079578453</v>
       </c>
     </row>
     <row r="107">
@@ -4058,10 +4058,10 @@
         <v>0.03793925388922854</v>
       </c>
       <c r="D107" t="n">
-        <v>0.03869669192524531</v>
+        <v>0.03869669192524532</v>
       </c>
       <c r="E107" t="n">
-        <v>0.0397070009689169</v>
+        <v>0.03970700096891691</v>
       </c>
       <c r="F107" t="n">
         <v>0.02802353300042233</v>
@@ -4070,13 +4070,13 @@
         <v>0.03769868381087125</v>
       </c>
       <c r="H107" t="n">
-        <v>0.03291698676237122</v>
+        <v>0.03291698676237124</v>
       </c>
       <c r="I107" t="n">
         <v>0.0237839708806508</v>
       </c>
       <c r="J107" t="n">
-        <v>0.02356127106796465</v>
+        <v>0.02356127106796466</v>
       </c>
     </row>
     <row r="108">
@@ -4107,10 +4107,10 @@
         <v>1.316758712373258</v>
       </c>
       <c r="I108" t="n">
-        <v>0.8487406085862316</v>
+        <v>0.8487406085862313</v>
       </c>
       <c r="J108" t="n">
-        <v>0.8136641741570476</v>
+        <v>0.8136641741570477</v>
       </c>
     </row>
     <row r="109">
@@ -4126,7 +4126,7 @@
         <v>0.07206746192771281</v>
       </c>
       <c r="D109" t="n">
-        <v>0.08368064460067066</v>
+        <v>0.08368064460067065</v>
       </c>
       <c r="E109" t="n">
         <v>0.03217509356562723</v>
@@ -4160,7 +4160,7 @@
         <v>0.7171099878918478</v>
       </c>
       <c r="D110" t="n">
-        <v>0.817847386373744</v>
+        <v>0.8178473863737441</v>
       </c>
       <c r="E110" t="n">
         <v>0.5390073555502188</v>
@@ -4169,13 +4169,13 @@
         <v>0.7740271705795116</v>
       </c>
       <c r="G110" t="n">
-        <v>0.9573450008550979</v>
+        <v>0.957345000855098</v>
       </c>
       <c r="H110" t="n">
         <v>0.9829265719310722</v>
       </c>
       <c r="I110" t="n">
-        <v>0.5571604311676975</v>
+        <v>0.5571604311676974</v>
       </c>
       <c r="J110" t="n">
         <v>0.6523785881508116</v>
@@ -4191,13 +4191,13 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>3.952421666004323</v>
+        <v>3.952421666004322</v>
       </c>
       <c r="D111" t="n">
-        <v>4.938063608108977</v>
+        <v>4.938063608108976</v>
       </c>
       <c r="E111" t="n">
-        <v>3.070851240784997</v>
+        <v>3.070851240784998</v>
       </c>
       <c r="F111" t="n">
         <v>4.389660285303012</v>
@@ -4212,7 +4212,7 @@
         <v>2.637419059217414</v>
       </c>
       <c r="J111" t="n">
-        <v>3.582464096055162</v>
+        <v>3.582464096055161</v>
       </c>
     </row>
     <row r="112">
@@ -4231,7 +4231,7 @@
         <v>0.8065859765484706</v>
       </c>
       <c r="E112" t="n">
-        <v>0.4214473357093588</v>
+        <v>0.4214473357093587</v>
       </c>
       <c r="F112" t="n">
         <v>0.615377157939534</v>
@@ -4243,10 +4243,10 @@
         <v>0.700216849589451</v>
       </c>
       <c r="I112" t="n">
-        <v>0.4516743596916466</v>
+        <v>0.4516743596916465</v>
       </c>
       <c r="J112" t="n">
-        <v>0.4761458562703815</v>
+        <v>0.4761458562703816</v>
       </c>
     </row>
     <row r="113">
@@ -4262,13 +4262,13 @@
         <v>0.08395742965637014</v>
       </c>
       <c r="D113" t="n">
-        <v>0.08212752369827389</v>
+        <v>0.0821275236982739</v>
       </c>
       <c r="E113" t="n">
-        <v>0.05900665227658688</v>
+        <v>0.05900665227658687</v>
       </c>
       <c r="F113" t="n">
-        <v>0.05051914470614071</v>
+        <v>0.05051914470614072</v>
       </c>
       <c r="G113" t="n">
         <v>0.07216786114310397</v>
@@ -4280,7 +4280,7 @@
         <v>0.04374775678838109</v>
       </c>
       <c r="J113" t="n">
-        <v>0.03849539825836883</v>
+        <v>0.03849539825836882</v>
       </c>
     </row>
     <row r="114">
@@ -4308,10 +4308,10 @@
         <v>0.1104988990643451</v>
       </c>
       <c r="H114" t="n">
-        <v>0.114816920639104</v>
+        <v>0.1148169206391039</v>
       </c>
       <c r="I114" t="n">
-        <v>0.0685715995837497</v>
+        <v>0.06857159958374971</v>
       </c>
       <c r="J114" t="n">
         <v>0.06769431409168301</v>
@@ -4339,16 +4339,16 @@
         <v>0.6955385631102619</v>
       </c>
       <c r="G115" t="n">
-        <v>0.8169565868647422</v>
+        <v>0.8169565868647419</v>
       </c>
       <c r="H115" t="n">
         <v>0.9270768516655752</v>
       </c>
       <c r="I115" t="n">
-        <v>0.5215268911944189</v>
+        <v>0.5215268911944188</v>
       </c>
       <c r="J115" t="n">
-        <v>0.5589340555997925</v>
+        <v>0.5589340555997924</v>
       </c>
     </row>
     <row r="116">
@@ -4367,7 +4367,7 @@
         <v>0.1671356572657079</v>
       </c>
       <c r="E116" t="n">
-        <v>0.08074307715757918</v>
+        <v>0.0807430771575792</v>
       </c>
       <c r="F116" t="n">
         <v>0.1191013284019713</v>
@@ -4404,13 +4404,13 @@
         <v>0.1748915459275882</v>
       </c>
       <c r="F117" t="n">
-        <v>0.3096264485804802</v>
+        <v>0.3096264485804803</v>
       </c>
       <c r="G117" t="n">
         <v>0.2068290727839418</v>
       </c>
       <c r="H117" t="n">
-        <v>0.2964946655329068</v>
+        <v>0.2964946655329069</v>
       </c>
       <c r="I117" t="n">
         <v>0.111526156776454</v>
@@ -4466,7 +4466,7 @@
         <v>1.670235599812682</v>
       </c>
       <c r="D119" t="n">
-        <v>1.854722215534065</v>
+        <v>1.854722215534064</v>
       </c>
       <c r="E119" t="n">
         <v>0.887752172818904</v>
@@ -4484,7 +4484,7 @@
         <v>0.8186878274341224</v>
       </c>
       <c r="J119" t="n">
-        <v>0.8267970425116496</v>
+        <v>0.8267970425116495</v>
       </c>
     </row>
     <row r="120">
@@ -4503,19 +4503,19 @@
         <v>81.05219158026499</v>
       </c>
       <c r="E120" t="n">
-        <v>53.51251879239247</v>
+        <v>53.51251879239246</v>
       </c>
       <c r="F120" t="n">
-        <v>39.66077298987022</v>
+        <v>39.66077298987021</v>
       </c>
       <c r="G120" t="n">
-        <v>57.56982819686368</v>
+        <v>57.56982819686367</v>
       </c>
       <c r="H120" t="n">
-        <v>61.63226993608347</v>
+        <v>61.63226993608345</v>
       </c>
       <c r="I120" t="n">
-        <v>35.19607595024726</v>
+        <v>35.19607595024725</v>
       </c>
       <c r="J120" t="n">
         <v>31.87976475355523</v>
@@ -4549,7 +4549,7 @@
         <v>0.0164338555021441</v>
       </c>
       <c r="I121" t="n">
-        <v>0.00918881355806289</v>
+        <v>0.009188813558062888</v>
       </c>
       <c r="J121" t="n">
         <v>0.009659336842494487</v>
@@ -4577,16 +4577,16 @@
         <v>0.04345606607444297</v>
       </c>
       <c r="G122" t="n">
-        <v>0.05373480344379532</v>
+        <v>0.05373480344379531</v>
       </c>
       <c r="H122" t="n">
         <v>0.05628118917363874</v>
       </c>
       <c r="I122" t="n">
-        <v>0.03093412283147595</v>
+        <v>0.03093412283147594</v>
       </c>
       <c r="J122" t="n">
-        <v>0.0350586018013061</v>
+        <v>0.03505860180130611</v>
       </c>
     </row>
     <row r="123">
@@ -4608,10 +4608,10 @@
         <v>0.4773460145565426</v>
       </c>
       <c r="F123" t="n">
-        <v>0.5888817738952307</v>
+        <v>0.5888817738952308</v>
       </c>
       <c r="G123" t="n">
-        <v>0.7940898229834973</v>
+        <v>0.7940898229834974</v>
       </c>
       <c r="H123" t="n">
         <v>0.8366351184717458</v>
@@ -4633,10 +4633,10 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>0.9928473343283523</v>
+        <v>0.9928473343283524</v>
       </c>
       <c r="D124" t="n">
-        <v>0.9647113502822957</v>
+        <v>0.9647113502822956</v>
       </c>
       <c r="E124" t="n">
         <v>0.2915488105133532</v>
@@ -4648,7 +4648,7 @@
         <v>0.8227710644108003</v>
       </c>
       <c r="H124" t="n">
-        <v>0.755940956591574</v>
+        <v>0.7559409565915741</v>
       </c>
       <c r="I124" t="n">
         <v>0.4185167578759832</v>
@@ -4701,7 +4701,7 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>0.4377205972432319</v>
+        <v>0.4377205972432318</v>
       </c>
       <c r="D126" t="n">
         <v>0.4473317930229601</v>
@@ -4744,16 +4744,16 @@
         <v>0.331793838272082</v>
       </c>
       <c r="F127" t="n">
-        <v>0.5277747378894979</v>
+        <v>0.527774737889498</v>
       </c>
       <c r="G127" t="n">
-        <v>0.6527540884412891</v>
+        <v>0.6527540884412892</v>
       </c>
       <c r="H127" t="n">
-        <v>0.732575293842731</v>
+        <v>0.7325752938427311</v>
       </c>
       <c r="I127" t="n">
-        <v>0.444662857663737</v>
+        <v>0.4446628576637369</v>
       </c>
       <c r="J127" t="n">
         <v>0.4126408411655091</v>
@@ -4874,7 +4874,7 @@
         <v>0.4049809720069281</v>
       </c>
       <c r="D131" t="n">
-        <v>0.3767191786281577</v>
+        <v>0.3767191786281576</v>
       </c>
       <c r="E131" t="n">
         <v>0.2094123945036249</v>
@@ -4892,7 +4892,7 @@
         <v>0.1563251352768341</v>
       </c>
       <c r="J131" t="n">
-        <v>0.1494311479443602</v>
+        <v>0.1494311479443601</v>
       </c>
     </row>
     <row r="132">
@@ -4942,7 +4942,7 @@
         <v>6.206407777253982</v>
       </c>
       <c r="D133" t="n">
-        <v>7.026606625058757</v>
+        <v>7.026606625058758</v>
       </c>
       <c r="E133" t="n">
         <v>1.939157446561349</v>
@@ -4951,10 +4951,10 @@
         <v>3.62384768188577</v>
       </c>
       <c r="G133" t="n">
-        <v>5.291570558900664</v>
+        <v>5.291570558900665</v>
       </c>
       <c r="H133" t="n">
-        <v>5.374482968330055</v>
+        <v>5.374482968330056</v>
       </c>
       <c r="I133" t="n">
         <v>2.904408933652301</v>
@@ -5013,10 +5013,10 @@
         <v>0.2287097807635124</v>
       </c>
       <c r="E135" t="n">
-        <v>0.04175644488510595</v>
+        <v>0.04175644488510594</v>
       </c>
       <c r="F135" t="n">
-        <v>0.04947160484073345</v>
+        <v>0.04947160484073346</v>
       </c>
       <c r="G135" t="n">
         <v>0.0975224805407954</v>
@@ -5028,7 +5028,7 @@
         <v>0.04972963067148637</v>
       </c>
       <c r="J135" t="n">
-        <v>0.04806202985997553</v>
+        <v>0.04806202985997554</v>
       </c>
     </row>
     <row r="136">
@@ -5062,7 +5062,7 @@
         <v>0.005871297986699622</v>
       </c>
       <c r="J136" t="n">
-        <v>0.005500527472471675</v>
+        <v>0.005500527472471674</v>
       </c>
     </row>
     <row r="137">
@@ -5121,10 +5121,10 @@
         <v>0.04068686981263041</v>
       </c>
       <c r="G138" t="n">
-        <v>0.05302468646513527</v>
+        <v>0.05302468646513528</v>
       </c>
       <c r="H138" t="n">
-        <v>0.05376350492866311</v>
+        <v>0.0537635049286631</v>
       </c>
       <c r="I138" t="n">
         <v>0.03202576049644099</v>
@@ -5143,25 +5143,25 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>0.03569303616075595</v>
+        <v>0.03569303616075594</v>
       </c>
       <c r="D139" t="n">
-        <v>0.03823982558354714</v>
+        <v>0.03823982558354715</v>
       </c>
       <c r="E139" t="n">
         <v>0.02384450346175599</v>
       </c>
       <c r="F139" t="n">
-        <v>0.03094254430702464</v>
+        <v>0.03094254430702463</v>
       </c>
       <c r="G139" t="n">
         <v>0.03810309305523307</v>
       </c>
       <c r="H139" t="n">
-        <v>0.04003425574187568</v>
+        <v>0.04003425574187567</v>
       </c>
       <c r="I139" t="n">
-        <v>0.02483623102659659</v>
+        <v>0.0248362310265966</v>
       </c>
       <c r="J139" t="n">
         <v>0.02368935833511291</v>

</xml_diff>